<commit_message>
Save library recording Instacart - 2a84c45b-1550-40de-92ab-8e237d462c1f - 2026-10-13T12:19:14.252787Z
</commit_message>
<xml_diff>
--- a/library/projects/qa-sample-app/recordings/2a84c45b-1550-40de-92ab-8e237d462c1f/resources/azure-devops.xlsx
+++ b/library/projects/qa-sample-app/recordings/2a84c45b-1550-40de-92ab-8e237d462c1f/resources/azure-devops.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,6 +448,585 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Open https://www.instacart.com/</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://www.instacart.com/</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Click Search</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>{"primary": "#search-bar-input", "x": 469, "y": 45, "text": "Search", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>step-002.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Type: Apple</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{"primary": "#search-bar-input"}</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>step-003.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Click 358,106</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>{"primary": "[data-testid=\"thumbnail\"]", "x": 358, "y": 106, "text": "", "tag": "img"}</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>step-004.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Click Safeway
+Delivery available
+Pickup available
+Groceries
+Bakery
+Deli
+Best seller
+Cu</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>{"primary": "#store-wrapper &gt; div:nth-of-type(1)", "x": 380, "y": 105, "text": "Safeway\nDelivery available\nPickup available\nGroceries\nBakery\nDeli\nBest seller\nCu", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>step-005.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Click 344,375</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>{"primary": "[data-testid=\"item-card-image\"]", "x": 344, "y": 375, "text": "", "tag": "img"}</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>step-006.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Click 364,371</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>{"primary": null, "x": 364, "y": 371, "text": null, "tag": null}</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>step-007.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Click Add to cart</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; div:nth-of-type(3) &gt; div:nth-of-type(2) &gt; button:nth-of-type(2) &gt; span:nth-of-type(1)", "x": 756, "y": 348, "text": "Add to cart", "tag": "span"}</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>step-008.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Click Item instructions</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(2) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; div:nth-of-type(4) &gt; div:nth-of-type(1) &gt; div:nth-of-type(1)", "x": 926, "y": 350, "text": "Item instructions", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>step-009.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Click Honeycrisp Apples
+About 0.5 lb each
+• $4.69 / lb
+Final cost by weight
+• In seaso</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>{"primary": "#item_details &gt; div:nth-of-type(2) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1)", "x": 563, "y": 326, "text": "Honeycrisp Apples\nAbout 0.5 lb each\n\u2022 $4.69 / lb\nFinal cost by weight\n\u2022 In seaso", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>step-010.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Click This is a carousel with one large image and a track of thumbnails. Select any of</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>{"primary": "#item_details &gt; div:nth-of-type(2)", "x": 369, "y": 326, "text": "This is a carousel with one large image and a track of thumbnails. Select any of", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>step-011.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Click Item instructions</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(2) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; div:nth-of-type(4) &gt; div:nth-of-type(1) &gt; div:nth-of-type(1)", "x": 802, "y": 337, "text": "Item instructions", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>step-012.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Click Add note for shopper</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(2) &gt; button:nth-of-type(1) &gt; span:nth-of-type(1) &gt; div:nth-of-type(1) &gt; div:nth-of-type(1) &gt; div:nth-of-type(1)", "x": 866, "y": 444, "text": "Add note for shopper", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>step-013.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Click Add instructions for ripeness, expiration dates, etc. (optional)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>{"primary": "#react-aria7633136552-_r_2_", "x": 305, "y": 299, "text": "Add instructions for ripeness, expiration dates, etc. (optional)", "tag": "textarea"}</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>step-014.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Click Add instructions for ripeness, expiration dates, etc. (optional)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>{"primary": "#react-aria7633136552-_r_2_", "x": 603, "y": 342, "text": "Add instructions for ripeness, expiration dates, etc. (optional)", "tag": "textarea"}</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>step-015.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Click Add instructions for ripeness, expiration dates, etc. (optional)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>{"primary": "#react-aria7633136552-_r_2_", "x": 537, "y": 314, "text": "Add instructions for ripeness, expiration dates, etc. (optional)", "tag": "textarea"}</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>step-016.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Click Add instructions for ripeness, expiration dates, etc. (optional)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>{"primary": "#react-aria7633136552-_r_2_", "x": 572, "y": 296, "text": "Add instructions for ripeness, expiration dates, etc. (optional)", "tag": "textarea"}</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>step-017.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Click Save note</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>{"primary": "#id-46 &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; button:nth-of-type(1)", "x": 607, "y": 439, "text": "Save note", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>step-018.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Click 314,321</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(1) &gt; div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(1) &gt; img:nth-of-type(1)", "x": 314, "y": 321, "text": "", "tag": "img"}</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>step-019.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Instacart</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Press Control+v</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Control+v</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>step-020.png</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>